<commit_message>
fix: apply three improvements to Codex B题 solution
1. Problem 3 bias decision: use F-test with engineering threshold (0.1m
   bias norm) instead of arbitrary heuristic thresholds (was 0.5m + 5%),
   correcting the decision to adopt the statistically significant bias
2. Bootstrap CI velocity centering: use raw velocity in linearized delta
   perturbation (was incorrectly using centered velocity)
3. Report text: update abstract, markdown, docx, and PDF reports to
   reflect the correct bias decision for Problem 3
4. result.xlsx: fix index bug in write_result_xlsx that caused
   misaligned writes when dataframe index was non-sequential
</commit_message>
<xml_diff>
--- a/outputs/estimates_summary.xlsx
+++ b/outputs/estimates_summary.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:R4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -441,60 +441,80 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
+          <t>delta_95%CI_lower_s</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>delta_95%CI_upper_s</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>方式1时间偏差_s</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>方式2时间偏差_s</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>方式2相对方式1系统偏差_x_m</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>方式2相对方式1系统偏差_y_m</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>是否判定存在系统偏差</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>F统计量</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>F检验p值</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>融合重叠时长_s</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>带偏差模型MSE</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>无偏差模型MSE</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>偏差模型误差下降比例</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>实际数据候选偏差_x_m</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>实际数据候选偏差_y_m</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>实际数据带偏差候选delta_s</t>
         </is>
@@ -511,30 +531,38 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>198.4317011716356</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
         <v>0</v>
       </c>
       <c r="F2" t="n">
+        <v>198.4317011716356</v>
+      </c>
+      <c r="G2" t="n">
         <v>0</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="H2" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>否</t>
         </is>
-      </c>
-      <c r="H2" t="n">
-        <v>700.3500011716355</v>
-      </c>
-      <c r="I2" t="n">
-        <v>3.118510501802297e-11</v>
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
-      <c r="L2" t="inlineStr"/>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="n">
+        <v>700.3500011716355</v>
+      </c>
+      <c r="M2" t="n">
+        <v>3.118510501802297e-11</v>
+      </c>
       <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr"/>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -544,81 +572,105 @@
         <v>50.54647182799437</v>
       </c>
       <c r="C3" t="n">
+        <v>50.54230323182355</v>
+      </c>
+      <c r="D3" t="n">
+        <v>50.54919660362494</v>
+      </c>
+      <c r="E3" t="n">
         <v>0</v>
       </c>
-      <c r="D3" t="n">
+      <c r="F3" t="n">
         <v>50.54647182799437</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>3.488432768569789</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>-1.822345826219965</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>是</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="J3" t="n">
+        <v>193895.5332775088</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.110223024625157e-16</v>
+      </c>
+      <c r="L3" t="n">
         <v>689.9754718279944</v>
       </c>
-      <c r="I3" t="n">
+      <c r="M3" t="n">
         <v>0.270622485362336</v>
       </c>
-      <c r="J3" t="n">
+      <c r="N3" t="n">
         <v>15.48445000528549</v>
       </c>
-      <c r="K3" t="n">
+      <c r="O3" t="n">
         <v>0.9825229513951118</v>
       </c>
-      <c r="L3" t="inlineStr"/>
-      <c r="M3" t="inlineStr"/>
-      <c r="N3" t="inlineStr"/>
+      <c r="P3" t="inlineStr"/>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
         <v>3</v>
       </c>
       <c r="B4" t="n">
-        <v>-367.8997979676832</v>
+        <v>-367.9066546706907</v>
       </c>
       <c r="C4" t="n">
-        <v>0</v>
+        <v>-367.9134909224867</v>
       </c>
       <c r="D4" t="n">
-        <v>-367.8997979676832</v>
+        <v>-367.9005427909877</v>
       </c>
       <c r="E4" t="n">
         <v>0</v>
       </c>
       <c r="F4" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>否</t>
-        </is>
+        <v>-367.9066546706907</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.1608413016526384</v>
       </c>
       <c r="H4" t="n">
-        <v>299.9797979676832</v>
-      </c>
-      <c r="I4" t="n">
+        <v>-0.1969062524867408</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>22.91616519328431</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.327221665903267e-10</v>
+      </c>
+      <c r="L4" t="n">
+        <v>299.9866546706907</v>
+      </c>
+      <c r="M4" t="n">
+        <v>3.758512706862233</v>
+      </c>
+      <c r="N4" t="n">
         <v>3.815971478090727</v>
       </c>
-      <c r="J4" t="n">
-        <v>3.815971478090727</v>
-      </c>
-      <c r="K4" t="n">
+      <c r="O4" t="n">
         <v>0.01505744253026827</v>
       </c>
-      <c r="L4" t="n">
+      <c r="P4" t="n">
         <v>-0.1608413016526384</v>
       </c>
-      <c r="M4" t="n">
+      <c r="Q4" t="n">
         <v>-0.1969062524867408</v>
       </c>
-      <c r="N4" t="n">
+      <c r="R4" t="n">
         <v>-367.9066546706907</v>
       </c>
     </row>

</xml_diff>